<commit_message>
Migrate Home, News, Who We Are and Expertise & Impact
- New blocks: cards-news-list, cards-article-grid; styled cards-tile,
  cards-feature, columns-media, breadcrumb-trail from the source site
- Global design: brand tokens, Montserrat stand-in for Gotham, 640px type
  scale, link hover, feature-grid section layout, section spacing
- Importer: home and news templates, parsers and import scripts;
  transformers extended for feature-grid and home/news cleanup

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-expertise-and-impact.report.xlsx
+++ b/tools/importer/reports/import-expertise-and-impact.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>_reportFile</t>
   </si>
@@ -49,13 +49,70 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-01T13:13:08.539Z</t>
+    <t>2026-10-28T10:59:13.510Z</t>
   </si>
   <si>
     <t>Expertise and impact | Kaiser Permanente</t>
   </si>
   <si>
     <t>https://about.kaiserpermanente.org/expertise-and-impact</t>
+  </si>
+  <si>
+    <t>index.report.json</t>
+  </si>
+  <si>
+    <t>["cards-tile","cards-tile","cards-feature","cards-news-list"]</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>home</t>
+  </si>
+  <si>
+    <t>2026-10-28T10:59:05.764Z</t>
+  </si>
+  <si>
+    <t>We’re transforming health and health care – find out how | Kaiser Permanente</t>
+  </si>
+  <si>
+    <t>https://about.kaiserpermanente.org/</t>
+  </si>
+  <si>
+    <t>news.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb-trail","cards-tile","cards-tile","cards-feature","cards-article-grid"]</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
+    <t>2026-10-28T10:58:37.063Z</t>
+  </si>
+  <si>
+    <t>News | Kaiser Permanente</t>
+  </si>
+  <si>
+    <t>https://about.kaiserpermanente.org/news</t>
+  </si>
+  <si>
+    <t>who-we-are.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb-trail","cards-tile","columns-media"]</t>
+  </si>
+  <si>
+    <t>who-we-are</t>
+  </si>
+  <si>
+    <t>2026-10-28T10:59:19.522Z</t>
+  </si>
+  <si>
+    <t>Who we are | Kaiser Permanente</t>
+  </si>
+  <si>
+    <t>https://about.kaiserpermanente.org/who-we-are</t>
   </si>
 </sst>
 </file>
@@ -444,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -452,8 +509,7 @@
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -506,6 +562,84 @@
       </c>
       <c r="H2" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>